<commit_message>
Rewrite national games project with the student's text analysis
Rebuilds the paper in the first person from the collected data: 11
works (4 tales, 7 epics), 16 episodes. Horse games dominate the epics,
games act as tests in tales and show the hero's qualities in epics, and
all four asyk episodes start the plot. Episode summaries derived from
the student's quotes fill the empty columns (tuzetuler.json). Survey
results stay as placeholders until the Google Forms export arrives.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWp2V469ega9rMmDw4DHEN
</commit_message>
<xml_diff>
--- a/Zerde_Ulttyq_oiyndar/Zertteu_kestesi.xlsx
+++ b/Zerde_Ulttyq_oiyndar/Zertteu_kestesi.xlsx
@@ -1332,7 +1332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1383,8 +1383,16 @@
           <t>Ертегі</t>
         </is>
       </c>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="7" t="n"/>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Ер Төстік [Мәтін] : қазақтың көне ертегілері (жаңартылған нұсқа) / М. Байбеков О. Байбеков ... – Тараз : Сенім, 2019</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -1400,8 +1408,16 @@
           <t>Ертегі</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="7" t="n"/>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>https://adebiportal.kz/kz/balaqai/view/kerqula-atty-kendebai__126</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -1417,8 +1433,16 @@
           <t>Ертегі</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="7" t="n"/>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Алтын сақа – Алматы, 1972.</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -1426,7 +1450,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Аяз би</t>
+          <t>Күн астындағы Күнікей қыз</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1434,8 +1458,16 @@
           <t>Ертегі</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="7" t="n"/>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>https://bilim-all.kz/article/263</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -1443,16 +1475,24 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Жиренше шешен</t>
+          <t>Алпамыс батыр</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Ертегі</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="7" t="n"/>
+          <t>Жыр</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Алпамыс батыр : эпостың баяны / ... – Астана : Фолиант, 2012.</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -1460,16 +1500,24 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Алдар Көсе әңгімелері</t>
+          <t>Қобыланды батыр</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Ертегі</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="7" t="n"/>
+          <t>Жыр</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Қобыланды батыр [Мәтін] / ... – Алматы : Mazmundama, 2022</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -1477,16 +1525,24 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Қаңбақ шал</t>
+          <t>Ер Тарғын</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Ертегі</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="7" t="n"/>
+          <t>Жыр</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Ер Тарғын [Мәтін] : батырлар жыры / ... – Астана : Алматыкітап, 2007.</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -1494,16 +1550,24 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Күн астындағы Күнікей қыз</t>
+          <t>Қамбар батыр</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ертегі</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="7" t="n"/>
+          <t>Жыр</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>https://bilim-all.kz/olen/4898-qambar-batyr</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -1511,7 +1575,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Алпамыс батыр</t>
+          <t>Қыз Жібек</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1519,8 +1583,16 @@
           <t>Жыр</t>
         </is>
       </c>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="7" t="n"/>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Қыз Жібек [Мәтін] : Лиро-эпостық поэма  – Алматы : Мектеп, 2003.</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -1528,7 +1600,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Қобыланды батыр</t>
+          <t>Қозы Көрпеш – Баян сұлу</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1536,8 +1608,16 @@
           <t>Жыр</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="7" t="n"/>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Қозы Көрпеш - Баян Сұлу [Мәтін] : лиро-эпостық поэма : М. Ж. Көпейұлы нұсқасы / ... – Алматы : Мектеп, 2006</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -1545,7 +1625,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Ер Тарғын</t>
+          <t>Айман – Шолпан</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1553,80 +1633,20 @@
           <t>Жыр</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="7" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Қамбар батыр</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Жыр</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="7" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Қыз Жібек</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Жыр</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="7" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Қозы Көрпеш – Баян сұлу</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Жыр</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="7" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Айман – Шолпан</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Жыр</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="7" t="n"/>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Айман-Шолпан [Мәтін] : Қазақ эпосы / ; Қазақ ССР Ғылым Академиясы, Тіл және әдебиет институты ; [баспаға даярлаған Ы. Т. Дүйсенбаев]... – Алматы : Қазақ ССР Ғылым Академиясының Баспасы, 1957</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>иә</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2 E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2 E3 E4 E5 E6 E7 E8 E9 E10 E11 E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"иә,жоқ"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1718,336 +1738,770 @@
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="n"/>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Алпамыс батыр</t>
+        </is>
+      </c>
       <c r="C2" s="4">
-        <f>IFERROR(VLOOKUP(B2,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D2" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B2,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Жамбы ату</t>
+        </is>
+      </c>
       <c r="E2" s="6" t="n"/>
       <c r="F2" s="5">
         <f>IFERROR(VLOOKUP(D2,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="7" t="n"/>
-      <c r="J2" s="6" t="n"/>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Алпамыс, Ұлтан</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Алпамыс бөгелген жоқ, садақты шірене тартып, жамбыны сыңғыр
+еткізіп атып түсірді.</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>С</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Ұлтан ханға барсам деп,
+Жамбыны атып алсам деп,
+Көңілі тасып, құлшынды.
+Анасымен көрісіп,
+Көздің жасын төгісіп,                                         Енді атына мінеді,
+Жамбыға қарай жүреді.                           «Диуана да келді!»— деп,
+Мазақ қып Ұлтан күледі.
+Атайын деп оқталып,
+Төсіне садақ тіреді.
+Атып тастап жамбыны,
+Ұлтанға жетіп келеді.</t>
+        </is>
+      </c>
       <c r="K2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="n"/>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Алпамыс батыр</t>
+        </is>
+      </c>
       <c r="C3" s="4">
-        <f>IFERROR(VLOOKUP(B3,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D3" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B3,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Көкпар</t>
+        </is>
+      </c>
       <c r="E3" s="6" t="n"/>
       <c r="F3" s="5">
         <f>IFERROR(VLOOKUP(D3,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="7" t="n"/>
-      <c r="J3" s="6" t="n"/>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Жәдігер, Гүлбаршын</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Жәдігер ойлады: «Менің көкпар шабатын заманым болса, өстіп жүрем бе, бұл көкпарды Қарлығаш апама апарып берейін, жігіттерге асып берсін!» — деп, мойнында кісен, аяғында шынжыр, құнан атына сүйретіп ауылға алып барды.</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Қ</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Гүлбаршынның алдына
+Көкпар әкеп тастады,
+Өңгеріп серке даладан.</t>
+        </is>
+      </c>
       <c r="K3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="n"/>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Қобыланды батыр</t>
+        </is>
+      </c>
       <c r="C4" s="4">
-        <f>IFERROR(VLOOKUP(B4,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D4" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B4,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Бәйге</t>
+        </is>
+      </c>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="5">
         <f>IFERROR(VLOOKUP(D4,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="6" t="n"/>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Құртқа, Қобыланды</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Бәйгеден келген аттар туралы айтылады; Құртқа Қобыландының сапарға аттанатынын біліп, Тайбурылға алтын ер салып дайындайды.</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Қ</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Бәйгеден келген кѳк дѳнен,
+Түнімен ұйқы кѳрмеген
+Қобландыдай батырдың
+Тоқтамасын білген соң,
+Тайбурылдың үстіне
+Алтыннан тұрман ер салып,
+Аз ғана азық, жем салып,
+Ақ орданың алдынан
+Ѳткізді Құртқа кѳлденең</t>
+        </is>
+      </c>
       <c r="K4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="n"/>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Ер Төстік</t>
+        </is>
+      </c>
       <c r="C5" s="4">
-        <f>IFERROR(VLOOKUP(B5,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D5" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B5,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Бәйге</t>
+        </is>
+      </c>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="5">
         <f>IFERROR(VLOOKUP(D5,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="6" t="n"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Ер Төстік, Темір хан</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Темір хан ат бәйгесін өткізіп, бар жүйрігін қосады; Төстік Шалқұйрықты бәйгеге дайындайды, аттар бір жұмалық жерден шабады.</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Қ</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Бұдан жеңілген соң Темір хан ат шабысына шығады. Өзінің бар жүйрігін бәйгеге қосады. Ер Төстік Шалқұйрықты даярлайды. Қарақшының түбіне келген соң, Шалқұйрыққа тіл бітеді: - Егер атты өте алысқа айдаса, менің шабысым өте жылдам болады. Үш күн шапсам, бүйірім қызып, өзімді тоқтатуға шамам келмей, кетіп қалуым мүмкін. Мен келе жатқанда алдымнан арқан керіп қой. Арқан үш қабат болсын, бір қабаты кендірден болсын. Үш қабат арқанның үшеуі де үзілсе, мен саған жоқпын, ағынымды тоқтата алмай кеткенім, үшеуі де үзілмесе, мен жығылып өлемін, онда да саған жоқпын. Егер арқан жартылай үзілсе, мен тоқтаймын, жығылып қалсам да, жаным қайтадан кіреді, күдер үзбе, - дейді. "Ер Төстіктің жалғыз шолағы бір жерде зарығып өліп қалсын!" - деп, Темір хан атты бір жұмалық жерге айдатады.Бір жеті өткен соң, бәйге аттары қайтып оралады. Темір хан мен Кеще хан балуан және ат бәйгесінен жеңіліп, не қыларын білмей, сасады. "Енді жаяу жарыс салып көрейік", - дейді.</t>
+        </is>
+      </c>
       <c r="K5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Ер Төстік</t>
+        </is>
+      </c>
       <c r="C6" s="4">
-        <f>IFERROR(VLOOKUP(B6,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D6" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B6,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Күрес</t>
+        </is>
+      </c>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="5">
         <f>IFERROR(VLOOKUP(D6,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="6" t="n"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Таусоғар, Темір хан</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Балуан күресінде жер астының алыптары Таусоғарға шақ келмейді, ол тауды көтеріп, күшін көрсетеді.</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>С</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Балуан күресі басталады. Таусоғарға балуан шақ келмейді. Жер астының алыптарының бәрі жығылып бітеді. Күресуге кісі шықпаған соң, Таусоғар бір тауды көтеріп алып, жұртқа күшін көрсетеді. Темір хан мен Кеще хан қатты сасып:
+     -Тауды біз жаққа қоя көрмесін! - деп Төстікке жалынады.</t>
+        </is>
+      </c>
       <c r="K6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="n"/>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Ер Төстік</t>
+        </is>
+      </c>
       <c r="C7" s="4">
-        <f>IFERROR(VLOOKUP(B7,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D7" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B7,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Асық</t>
+        </is>
+      </c>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="5">
         <f>IFERROR(VLOOKUP(D7,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="6" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Ер Төстік</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Төстік асық ойнап жүріп, кемпірдің баласын ұрып қалады; кемпірдің ызасынан кейін Төстік ағаларын іздеп жолға шығады.</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Б</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Тағы бір күні Төстік асық ойнап жүріп, әлгі кемпірдің жалғыз баласын жұдырығымен қойып жіберсе, бала талып қалады.</t>
+        </is>
+      </c>
       <c r="K7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="n"/>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Керқұла атты Кендебай</t>
+        </is>
+      </c>
       <c r="C8" s="4">
-        <f>IFERROR(VLOOKUP(B8,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D8" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B8,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Күрес</t>
+        </is>
+      </c>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="5">
         <f>IFERROR(VLOOKUP(D8,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="6" t="n"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Кендебай</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Кендебай ерекше күшті болып өседі: күрескенін жыға береді, құдыққа құлаған түйелерді жалғыз тартып шығарады.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Б</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>Сондай күшті болыпты, алысқанын алып ұра беріпті, күрескенін жыға беріпті, шыңырау құдыққа құлаған атандарды жалғыз тартып шығара беріпті.</t>
+        </is>
+      </c>
       <c r="K8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="n"/>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Алтын сақа</t>
+        </is>
+      </c>
       <c r="C9" s="4">
-        <f>IFERROR(VLOOKUP(B9,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D9" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B9,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Асық</t>
+        </is>
+      </c>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="5">
         <f>IFERROR(VLOOKUP(D9,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="6" t="n"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Бала, жалмауыз кемпір</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Ауыл көшкенде баланың алтын сақасы жұртта қалады; бала оны алуға қайтып барып, жалмауыз кемпірге кездеседі.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Б</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>Сонымен бай жалмауыз кемпірге уәдесін беріп, жылқыларын айдап, кетіп қалады. Ертеңінде көшеді, жалғыз баласының алтын сақасын ұмыттырып, жұртқа тастап кетеді. Ауыл жаңа қонысқа көшіп барады. Асық ойнайын десе, сақасы жоқ, бала алтын сақасын жоқтап, жылайды. Жұртқа келсе, алтын сақасы ошақ басындағы тезек түбінде жатыр екен. Сақа жанында бір кемпір отыр екен. Бала кемпірге:
+— Шеше, анау жатқан сақамды алып берші! – дейді.
+Сонда кемпір:
+— Шырағым, өзің түсіп ал. Кәріліктен отырсам -тұра алмаймын, тұрсам - отыра алмаймын, – дейді.</t>
+        </is>
+      </c>
       <c r="K9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="n"/>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Қыз Жібек</t>
+        </is>
+      </c>
       <c r="C10" s="4">
-        <f>IFERROR(VLOOKUP(B10,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D10" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B10,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Асық</t>
+        </is>
+      </c>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="5">
         <f>IFERROR(VLOOKUP(D10,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="6" t="n"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Жастар</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Жастардың қызықты өмірі суреттеледі: олар тай-құлындай тебісіп, асық ойнап алысады.</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Б</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Көп қызыққа батысқан, Тай құлындай тебіскен, Асық ойнап алысқан.</t>
+        </is>
+      </c>
       <c r="K10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="n"/>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Күн астындағы Күнікей қыз</t>
+        </is>
+      </c>
       <c r="C11" s="4">
-        <f>IFERROR(VLOOKUP(B11,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B11,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Басқа</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Жаяу бәйге</t>
+        </is>
+      </c>
       <c r="F11" s="5">
         <f>IFERROR(VLOOKUP(D11,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Бала, мыстан кемпір, хан</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Хан сөзінен танып, қызын жаяу бәйгеде озған адамға беретінін айтады; ханның жағынан жүйрік мыстан кемпір шығады.</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>С</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Бірақ, хан сөзінен танып, бұл жолы қызын бермей:
+— Енді жаяу бәйгеден озып келгенге беремін, – дейді. Жаяу бәйгеге ханның елінен бір жүйрік мыстан кемпір шығады.</t>
+        </is>
+      </c>
       <c r="K11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="n"/>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Күн астындағы Күнікей қыз</t>
+        </is>
+      </c>
       <c r="C12" s="4">
-        <f>IFERROR(VLOOKUP(B12,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D12" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B12,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Күрес</t>
+        </is>
+      </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="5">
         <f>IFERROR(VLOOKUP(D12,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Дәу, өгіз балуан, хан</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Хан қызын күресте жеңгенге беремін дейді; баланың жолдасы – екі қолына екі тау ұстаған дәу – ханның балуанын жығады.</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>С</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Хан ертеңіне, ел-жұртын жиып, балуан күрестіреді. Осы топта кімде-кім күресіп жығып, күші асса, қызымды соған беремін, – дейді. Ханның елі жағынан бір өгіз балуан шығады. Бала жағынан екі қолына екі тау ұстап жүруші дәу шығады. Екі балуан күресіп, дәу жығып кетеді.</t>
+        </is>
+      </c>
       <c r="K12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="n"/>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Ер Тарғын</t>
+        </is>
+      </c>
       <c r="C13" s="4">
-        <f>IFERROR(VLOOKUP(B13,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D13" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B13,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Бәйге</t>
+        </is>
+      </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="5">
         <f>IFERROR(VLOOKUP(D13,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Ер Тарғын</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Тарғын Тарлан атымен жауға шабуды «Тарлан бәйгесі» деп атайды – бәйге бейнесі батырдың ерлігін көрсетеді.</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Қ</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>Кебеже қарын, кең құрсақ,
+Құлжа мойын төгерек,
+Ұмтыла шапқан Тарланым,
+Алты мыңдай кісі екен,
+Тіл жіберсең саған серт!
+Сен желігіп жүргенде,
+Таяна шапса маған серт!
+Тауыса шапса бұ жауды,
+Сонда бітер Тарлан бәйгесі</t>
+        </is>
+      </c>
       <c r="K13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="6" t="n"/>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Қамбар батыр</t>
+        </is>
+      </c>
       <c r="C14" s="4">
-        <f>IFERROR(VLOOKUP(B14,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D14" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B14,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Аударыспақ</t>
+        </is>
+      </c>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="5">
         <f>IFERROR(VLOOKUP(D14,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Қараман, бектер</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Қараман бастаған бектер кернейлетіп қаладан шығып, ат үстінде аударысып ойнайды.</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Қ</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>Қараман шықты қаладан,
+Кернейлері бақылдап,
+Байрақтар тулап көтерген,
+Алтыннан қалқан жарқылдап,
+Сыбызғы, сырнай шақылдап,
+Мінгендері дәл бедеу,
+Келеді бектер дабылдап.
+Аударысып ойнайды
+Буыршындай тақымдап;</t>
+        </is>
+      </c>
       <c r="K14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="6" t="n"/>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Қозы Көрпеш – Баян сұлу</t>
+        </is>
+      </c>
       <c r="C15" s="4">
-        <f>IFERROR(VLOOKUP(B15,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D15" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B15,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Аударыспақ</t>
+        </is>
+      </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="5">
         <f>IFERROR(VLOOKUP(D15,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="7" t="n"/>
-      <c r="J15" s="6" t="n"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Қозы Көрпеш</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Қозы жылқы бағып жүріп, тоқсан құлмен аударыспақ ойнайды және бәрін аттан аударып түсіреді – оның алып күші көрінеді.</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Б</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>Қарабай оны жақсы көріп, жылқы бағуға жұмсайды. Қозы алғашқыда Қодармен әзілдесіп, кейде ойнап, ат үстінен жұлып алып жүреді. Кейде тоқсан құлмен аударыспақ ойнап, оларды тегісімен топырлатып жүреді. Халық ақындары бұл жерде Қозы Көрпешті жойқын алып түрінде суреттеп, оның жеңбейтін адамы жоқ деп сипаттайды.</t>
+        </is>
+      </c>
       <c r="K15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="6" t="n"/>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Қозы Көрпеш – Баян сұлу</t>
+        </is>
+      </c>
       <c r="C16" s="4">
-        <f>IFERROR(VLOOKUP(B16,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D16" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B16,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Асық</t>
+        </is>
+      </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="5">
         <f>IFERROR(VLOOKUP(D16,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="7" t="n"/>
-      <c r="J16" s="6" t="n"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Қозы Көрпеш, тазша бала</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Қозы бала күнін асық ойнап өткізеді; тазша баланың сақасын тартып алғанда, «жарыңды іздеп тапсайшы» деген сөз естиді.</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Б</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>Әкесінен жетім қалған Қозы Көрпеш ақылды анасы мен кемеңгер ағаларының қолында еркін өседі. Бала күнін бірыңғай асық ойнаумен өткізеді.Тазша баланың сақасын тартып алып, оның аузынан: «Менің сақамды тартып алғанша, жарыңды іздеп тапсайшы» деген сөз естиді.</t>
+        </is>
+      </c>
       <c r="K16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="n"/>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Айман – Шолпан</t>
+        </is>
+      </c>
       <c r="C17" s="4">
-        <f>IFERROR(VLOOKUP(B17,Шығармалар!$B$2:$C$16,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D17" s="6" t="n"/>
+        <f>IFERROR(VLOOKUP(B17,Шығармалар!$B$2:$C$12,2,0),"")</f>
+        <v/>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Бәйге</t>
+        </is>
+      </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="5">
         <f>IFERROR(VLOOKUP(D17,Ойындар!$B$2:$C$14,2,0),"")</f>
         <v/>
       </c>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="6" t="n"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Басыбар</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Басыбар бәйгеге ат жөнелтіп, қайта келетінін айтады – бәйге ас пен той дайындығының бөлігі ретінде аталады.</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>Қ</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>Басыбар: Тәйт, жоғал, ондайынды жолымнан ал
+былай! Күмілжімей, тек көмейің күлкілдемей сертінде қал
+жалтақтамай. Байлауым сол, кәзір бәйгеге ат жөнелтіп қайта
+мұнда келемін. Мыжымай қарсы алуға қамдана бер осы
+үйде!</t>
+        </is>
+      </c>
       <c r="K17" s="7" t="n"/>
     </row>
     <row r="18">
@@ -2056,7 +2510,7 @@
       </c>
       <c r="B18" s="6" t="n"/>
       <c r="C18" s="4">
-        <f>IFERROR(VLOOKUP(B18,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B18,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D18" s="6" t="n"/>
@@ -2077,7 +2531,7 @@
       </c>
       <c r="B19" s="6" t="n"/>
       <c r="C19" s="4">
-        <f>IFERROR(VLOOKUP(B19,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B19,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D19" s="6" t="n"/>
@@ -2098,7 +2552,7 @@
       </c>
       <c r="B20" s="6" t="n"/>
       <c r="C20" s="4">
-        <f>IFERROR(VLOOKUP(B20,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B20,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D20" s="6" t="n"/>
@@ -2119,7 +2573,7 @@
       </c>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="4">
-        <f>IFERROR(VLOOKUP(B21,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B21,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D21" s="6" t="n"/>
@@ -2140,7 +2594,7 @@
       </c>
       <c r="B22" s="6" t="n"/>
       <c r="C22" s="4">
-        <f>IFERROR(VLOOKUP(B22,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B22,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D22" s="6" t="n"/>
@@ -2161,7 +2615,7 @@
       </c>
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="4">
-        <f>IFERROR(VLOOKUP(B23,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B23,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D23" s="6" t="n"/>
@@ -2182,7 +2636,7 @@
       </c>
       <c r="B24" s="6" t="n"/>
       <c r="C24" s="4">
-        <f>IFERROR(VLOOKUP(B24,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B24,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D24" s="6" t="n"/>
@@ -2203,7 +2657,7 @@
       </c>
       <c r="B25" s="6" t="n"/>
       <c r="C25" s="4">
-        <f>IFERROR(VLOOKUP(B25,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B25,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D25" s="6" t="n"/>
@@ -2224,7 +2678,7 @@
       </c>
       <c r="B26" s="6" t="n"/>
       <c r="C26" s="4">
-        <f>IFERROR(VLOOKUP(B26,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B26,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D26" s="6" t="n"/>
@@ -2245,7 +2699,7 @@
       </c>
       <c r="B27" s="6" t="n"/>
       <c r="C27" s="4">
-        <f>IFERROR(VLOOKUP(B27,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B27,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D27" s="6" t="n"/>
@@ -2266,7 +2720,7 @@
       </c>
       <c r="B28" s="6" t="n"/>
       <c r="C28" s="4">
-        <f>IFERROR(VLOOKUP(B28,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B28,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D28" s="6" t="n"/>
@@ -2287,7 +2741,7 @@
       </c>
       <c r="B29" s="6" t="n"/>
       <c r="C29" s="4">
-        <f>IFERROR(VLOOKUP(B29,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B29,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D29" s="6" t="n"/>
@@ -2308,7 +2762,7 @@
       </c>
       <c r="B30" s="6" t="n"/>
       <c r="C30" s="4">
-        <f>IFERROR(VLOOKUP(B30,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B30,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D30" s="6" t="n"/>
@@ -2329,7 +2783,7 @@
       </c>
       <c r="B31" s="6" t="n"/>
       <c r="C31" s="4">
-        <f>IFERROR(VLOOKUP(B31,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B31,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D31" s="6" t="n"/>
@@ -2350,7 +2804,7 @@
       </c>
       <c r="B32" s="6" t="n"/>
       <c r="C32" s="4">
-        <f>IFERROR(VLOOKUP(B32,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B32,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D32" s="6" t="n"/>
@@ -2371,7 +2825,7 @@
       </c>
       <c r="B33" s="6" t="n"/>
       <c r="C33" s="4">
-        <f>IFERROR(VLOOKUP(B33,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B33,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D33" s="6" t="n"/>
@@ -2392,7 +2846,7 @@
       </c>
       <c r="B34" s="6" t="n"/>
       <c r="C34" s="4">
-        <f>IFERROR(VLOOKUP(B34,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B34,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D34" s="6" t="n"/>
@@ -2413,7 +2867,7 @@
       </c>
       <c r="B35" s="6" t="n"/>
       <c r="C35" s="4">
-        <f>IFERROR(VLOOKUP(B35,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B35,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D35" s="6" t="n"/>
@@ -2434,7 +2888,7 @@
       </c>
       <c r="B36" s="6" t="n"/>
       <c r="C36" s="4">
-        <f>IFERROR(VLOOKUP(B36,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B36,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D36" s="6" t="n"/>
@@ -2455,7 +2909,7 @@
       </c>
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="4">
-        <f>IFERROR(VLOOKUP(B37,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B37,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D37" s="6" t="n"/>
@@ -2476,7 +2930,7 @@
       </c>
       <c r="B38" s="6" t="n"/>
       <c r="C38" s="4">
-        <f>IFERROR(VLOOKUP(B38,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B38,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D38" s="6" t="n"/>
@@ -2497,7 +2951,7 @@
       </c>
       <c r="B39" s="6" t="n"/>
       <c r="C39" s="4">
-        <f>IFERROR(VLOOKUP(B39,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B39,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D39" s="6" t="n"/>
@@ -2518,7 +2972,7 @@
       </c>
       <c r="B40" s="6" t="n"/>
       <c r="C40" s="4">
-        <f>IFERROR(VLOOKUP(B40,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B40,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D40" s="6" t="n"/>
@@ -2539,7 +2993,7 @@
       </c>
       <c r="B41" s="6" t="n"/>
       <c r="C41" s="4">
-        <f>IFERROR(VLOOKUP(B41,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B41,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D41" s="6" t="n"/>
@@ -2560,7 +3014,7 @@
       </c>
       <c r="B42" s="6" t="n"/>
       <c r="C42" s="4">
-        <f>IFERROR(VLOOKUP(B42,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B42,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D42" s="6" t="n"/>
@@ -2581,7 +3035,7 @@
       </c>
       <c r="B43" s="6" t="n"/>
       <c r="C43" s="4">
-        <f>IFERROR(VLOOKUP(B43,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B43,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D43" s="6" t="n"/>
@@ -2602,7 +3056,7 @@
       </c>
       <c r="B44" s="6" t="n"/>
       <c r="C44" s="4">
-        <f>IFERROR(VLOOKUP(B44,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B44,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D44" s="6" t="n"/>
@@ -2623,7 +3077,7 @@
       </c>
       <c r="B45" s="6" t="n"/>
       <c r="C45" s="4">
-        <f>IFERROR(VLOOKUP(B45,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B45,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D45" s="6" t="n"/>
@@ -2644,7 +3098,7 @@
       </c>
       <c r="B46" s="6" t="n"/>
       <c r="C46" s="4">
-        <f>IFERROR(VLOOKUP(B46,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B46,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D46" s="6" t="n"/>
@@ -2665,7 +3119,7 @@
       </c>
       <c r="B47" s="6" t="n"/>
       <c r="C47" s="4">
-        <f>IFERROR(VLOOKUP(B47,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B47,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D47" s="6" t="n"/>
@@ -2686,7 +3140,7 @@
       </c>
       <c r="B48" s="6" t="n"/>
       <c r="C48" s="4">
-        <f>IFERROR(VLOOKUP(B48,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B48,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D48" s="6" t="n"/>
@@ -2707,7 +3161,7 @@
       </c>
       <c r="B49" s="6" t="n"/>
       <c r="C49" s="4">
-        <f>IFERROR(VLOOKUP(B49,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B49,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D49" s="6" t="n"/>
@@ -2728,7 +3182,7 @@
       </c>
       <c r="B50" s="6" t="n"/>
       <c r="C50" s="4">
-        <f>IFERROR(VLOOKUP(B50,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B50,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D50" s="6" t="n"/>
@@ -2749,7 +3203,7 @@
       </c>
       <c r="B51" s="6" t="n"/>
       <c r="C51" s="4">
-        <f>IFERROR(VLOOKUP(B51,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B51,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D51" s="6" t="n"/>
@@ -2770,7 +3224,7 @@
       </c>
       <c r="B52" s="6" t="n"/>
       <c r="C52" s="4">
-        <f>IFERROR(VLOOKUP(B52,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B52,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D52" s="6" t="n"/>
@@ -2791,7 +3245,7 @@
       </c>
       <c r="B53" s="6" t="n"/>
       <c r="C53" s="4">
-        <f>IFERROR(VLOOKUP(B53,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B53,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D53" s="6" t="n"/>
@@ -2812,7 +3266,7 @@
       </c>
       <c r="B54" s="6" t="n"/>
       <c r="C54" s="4">
-        <f>IFERROR(VLOOKUP(B54,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B54,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D54" s="6" t="n"/>
@@ -2833,7 +3287,7 @@
       </c>
       <c r="B55" s="6" t="n"/>
       <c r="C55" s="4">
-        <f>IFERROR(VLOOKUP(B55,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B55,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D55" s="6" t="n"/>
@@ -2854,7 +3308,7 @@
       </c>
       <c r="B56" s="6" t="n"/>
       <c r="C56" s="4">
-        <f>IFERROR(VLOOKUP(B56,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B56,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D56" s="6" t="n"/>
@@ -2875,7 +3329,7 @@
       </c>
       <c r="B57" s="6" t="n"/>
       <c r="C57" s="4">
-        <f>IFERROR(VLOOKUP(B57,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B57,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D57" s="6" t="n"/>
@@ -2896,7 +3350,7 @@
       </c>
       <c r="B58" s="6" t="n"/>
       <c r="C58" s="4">
-        <f>IFERROR(VLOOKUP(B58,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B58,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D58" s="6" t="n"/>
@@ -2917,7 +3371,7 @@
       </c>
       <c r="B59" s="6" t="n"/>
       <c r="C59" s="4">
-        <f>IFERROR(VLOOKUP(B59,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B59,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D59" s="6" t="n"/>
@@ -2938,7 +3392,7 @@
       </c>
       <c r="B60" s="6" t="n"/>
       <c r="C60" s="4">
-        <f>IFERROR(VLOOKUP(B60,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B60,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D60" s="6" t="n"/>
@@ -2959,7 +3413,7 @@
       </c>
       <c r="B61" s="6" t="n"/>
       <c r="C61" s="4">
-        <f>IFERROR(VLOOKUP(B61,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B61,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D61" s="6" t="n"/>
@@ -2980,7 +3434,7 @@
       </c>
       <c r="B62" s="6" t="n"/>
       <c r="C62" s="4">
-        <f>IFERROR(VLOOKUP(B62,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B62,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D62" s="6" t="n"/>
@@ -3001,7 +3455,7 @@
       </c>
       <c r="B63" s="6" t="n"/>
       <c r="C63" s="4">
-        <f>IFERROR(VLOOKUP(B63,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B63,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D63" s="6" t="n"/>
@@ -3022,7 +3476,7 @@
       </c>
       <c r="B64" s="6" t="n"/>
       <c r="C64" s="4">
-        <f>IFERROR(VLOOKUP(B64,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B64,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D64" s="6" t="n"/>
@@ -3043,7 +3497,7 @@
       </c>
       <c r="B65" s="6" t="n"/>
       <c r="C65" s="4">
-        <f>IFERROR(VLOOKUP(B65,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B65,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D65" s="6" t="n"/>
@@ -3064,7 +3518,7 @@
       </c>
       <c r="B66" s="6" t="n"/>
       <c r="C66" s="4">
-        <f>IFERROR(VLOOKUP(B66,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B66,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D66" s="6" t="n"/>
@@ -3085,7 +3539,7 @@
       </c>
       <c r="B67" s="6" t="n"/>
       <c r="C67" s="4">
-        <f>IFERROR(VLOOKUP(B67,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B67,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D67" s="6" t="n"/>
@@ -3106,7 +3560,7 @@
       </c>
       <c r="B68" s="6" t="n"/>
       <c r="C68" s="4">
-        <f>IFERROR(VLOOKUP(B68,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B68,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D68" s="6" t="n"/>
@@ -3127,7 +3581,7 @@
       </c>
       <c r="B69" s="6" t="n"/>
       <c r="C69" s="4">
-        <f>IFERROR(VLOOKUP(B69,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B69,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D69" s="6" t="n"/>
@@ -3148,7 +3602,7 @@
       </c>
       <c r="B70" s="6" t="n"/>
       <c r="C70" s="4">
-        <f>IFERROR(VLOOKUP(B70,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B70,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D70" s="6" t="n"/>
@@ -3169,7 +3623,7 @@
       </c>
       <c r="B71" s="6" t="n"/>
       <c r="C71" s="4">
-        <f>IFERROR(VLOOKUP(B71,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B71,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D71" s="6" t="n"/>
@@ -3190,7 +3644,7 @@
       </c>
       <c r="B72" s="6" t="n"/>
       <c r="C72" s="4">
-        <f>IFERROR(VLOOKUP(B72,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B72,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D72" s="6" t="n"/>
@@ -3211,7 +3665,7 @@
       </c>
       <c r="B73" s="6" t="n"/>
       <c r="C73" s="4">
-        <f>IFERROR(VLOOKUP(B73,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B73,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D73" s="6" t="n"/>
@@ -3232,7 +3686,7 @@
       </c>
       <c r="B74" s="6" t="n"/>
       <c r="C74" s="4">
-        <f>IFERROR(VLOOKUP(B74,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B74,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D74" s="6" t="n"/>
@@ -3253,7 +3707,7 @@
       </c>
       <c r="B75" s="6" t="n"/>
       <c r="C75" s="4">
-        <f>IFERROR(VLOOKUP(B75,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B75,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D75" s="6" t="n"/>
@@ -3274,7 +3728,7 @@
       </c>
       <c r="B76" s="6" t="n"/>
       <c r="C76" s="4">
-        <f>IFERROR(VLOOKUP(B76,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B76,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D76" s="6" t="n"/>
@@ -3295,7 +3749,7 @@
       </c>
       <c r="B77" s="6" t="n"/>
       <c r="C77" s="4">
-        <f>IFERROR(VLOOKUP(B77,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B77,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D77" s="6" t="n"/>
@@ -3316,7 +3770,7 @@
       </c>
       <c r="B78" s="6" t="n"/>
       <c r="C78" s="4">
-        <f>IFERROR(VLOOKUP(B78,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B78,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D78" s="6" t="n"/>
@@ -3337,7 +3791,7 @@
       </c>
       <c r="B79" s="6" t="n"/>
       <c r="C79" s="4">
-        <f>IFERROR(VLOOKUP(B79,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B79,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D79" s="6" t="n"/>
@@ -3358,7 +3812,7 @@
       </c>
       <c r="B80" s="6" t="n"/>
       <c r="C80" s="4">
-        <f>IFERROR(VLOOKUP(B80,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B80,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D80" s="6" t="n"/>
@@ -3379,7 +3833,7 @@
       </c>
       <c r="B81" s="6" t="n"/>
       <c r="C81" s="4">
-        <f>IFERROR(VLOOKUP(B81,Шығармалар!$B$2:$C$16,2,0),"")</f>
+        <f>IFERROR(VLOOKUP(B81,Шығармалар!$B$2:$C$12,2,0),"")</f>
         <v/>
       </c>
       <c r="D81" s="6" t="n"/>
@@ -3397,7 +3851,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="B2 B3 B4 B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20 B21 B22 B23 B24 B25 B26 B27 B28 B29 B30 B31 B32 B33 B34 B35 B36 B37 B38 B39 B40 B41 B42 B43 B44 B45 B46 B47 B48 B49 B50 B51 B52 B53 B54 B55 B56 B57 B58 B59 B60 B61 B62 B63 B64 B65 B66 B67 B68 B69 B70 B71 B72 B73 B74 B75 B76 B77 B78 B79 B80 B81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Шығармалар!$B$2:$B$16</formula1>
+      <formula1>=Шығармалар!$B$2:$B$12</formula1>
     </dataValidation>
     <dataValidation sqref="D2 D3 D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Ойындар!$B$2:$B$14</formula1>

</xml_diff>

<commit_message>
Add survey results and work editions to the national games project
Import 19 consented Google Forms responses into the research workbook,
write the survey section from them, and list the editions the student
read in table 3 and the references.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWp2V469ega9rMmDw4DHEN
</commit_message>
<xml_diff>
--- a/Zerde_Ulttyq_oiyndar/Zertteu_kestesi.xlsx
+++ b/Zerde_Ulttyq_oiyndar/Zertteu_kestesi.xlsx
@@ -4040,31 +4040,81 @@
           <t>С01</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n"/>
-      <c r="C2" s="7" t="n"/>
-      <c r="D2" s="7" t="n"/>
-      <c r="E2" s="7" t="n"/>
-      <c r="F2" s="7" t="n"/>
-      <c r="G2" s="7" t="n"/>
-      <c r="H2" s="7" t="n"/>
-      <c r="I2" s="7" t="n"/>
-      <c r="J2" s="7" t="n"/>
-      <c r="K2" s="7" t="n"/>
-      <c r="L2" s="7" t="n"/>
-      <c r="M2" s="7" t="n"/>
-      <c r="N2" s="7" t="n"/>
-      <c r="O2" s="7" t="n"/>
-      <c r="P2" s="7" t="n"/>
-      <c r="Q2" s="7" t="n"/>
-      <c r="R2" s="7" t="n"/>
-      <c r="S2" s="7" t="n"/>
-      <c r="T2" s="7" t="n"/>
-      <c r="U2" s="7" t="n"/>
-      <c r="V2" s="7" t="n"/>
-      <c r="W2" s="7" t="n"/>
-      <c r="X2" s="7" t="n"/>
-      <c r="Y2" s="7" t="n"/>
-      <c r="Z2" s="7" t="n"/>
+      <c r="B2" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z2" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -4072,31 +4122,81 @@
           <t>С02</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n"/>
-      <c r="C3" s="7" t="n"/>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="7" t="n"/>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="7" t="n"/>
-      <c r="H3" s="7" t="n"/>
-      <c r="I3" s="7" t="n"/>
-      <c r="J3" s="7" t="n"/>
-      <c r="K3" s="7" t="n"/>
-      <c r="L3" s="7" t="n"/>
-      <c r="M3" s="7" t="n"/>
-      <c r="N3" s="7" t="n"/>
-      <c r="O3" s="7" t="n"/>
-      <c r="P3" s="7" t="n"/>
-      <c r="Q3" s="7" t="n"/>
-      <c r="R3" s="7" t="n"/>
-      <c r="S3" s="7" t="n"/>
-      <c r="T3" s="7" t="n"/>
-      <c r="U3" s="7" t="n"/>
-      <c r="V3" s="7" t="n"/>
-      <c r="W3" s="7" t="n"/>
-      <c r="X3" s="7" t="n"/>
-      <c r="Y3" s="7" t="n"/>
-      <c r="Z3" s="7" t="n"/>
+      <c r="B3" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z3" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -4104,31 +4204,81 @@
           <t>С03</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="7" t="n"/>
-      <c r="P4" s="7" t="n"/>
-      <c r="Q4" s="7" t="n"/>
-      <c r="R4" s="7" t="n"/>
-      <c r="S4" s="7" t="n"/>
-      <c r="T4" s="7" t="n"/>
-      <c r="U4" s="7" t="n"/>
-      <c r="V4" s="7" t="n"/>
-      <c r="W4" s="7" t="n"/>
-      <c r="X4" s="7" t="n"/>
-      <c r="Y4" s="7" t="n"/>
-      <c r="Z4" s="7" t="n"/>
+      <c r="B4" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z4" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -4136,31 +4286,81 @@
           <t>С04</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="7" t="n"/>
-      <c r="N5" s="7" t="n"/>
-      <c r="O5" s="7" t="n"/>
-      <c r="P5" s="7" t="n"/>
-      <c r="Q5" s="7" t="n"/>
-      <c r="R5" s="7" t="n"/>
-      <c r="S5" s="7" t="n"/>
-      <c r="T5" s="7" t="n"/>
-      <c r="U5" s="7" t="n"/>
-      <c r="V5" s="7" t="n"/>
-      <c r="W5" s="7" t="n"/>
-      <c r="X5" s="7" t="n"/>
-      <c r="Y5" s="7" t="n"/>
-      <c r="Z5" s="7" t="n"/>
+      <c r="B5" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="T5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z5" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -4168,31 +4368,81 @@
           <t>С05</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="7" t="n"/>
-      <c r="N6" s="7" t="n"/>
-      <c r="O6" s="7" t="n"/>
-      <c r="P6" s="7" t="n"/>
-      <c r="Q6" s="7" t="n"/>
-      <c r="R6" s="7" t="n"/>
-      <c r="S6" s="7" t="n"/>
-      <c r="T6" s="7" t="n"/>
-      <c r="U6" s="7" t="n"/>
-      <c r="V6" s="7" t="n"/>
-      <c r="W6" s="7" t="n"/>
-      <c r="X6" s="7" t="n"/>
-      <c r="Y6" s="7" t="n"/>
-      <c r="Z6" s="7" t="n"/>
+      <c r="B6" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -4200,31 +4450,81 @@
           <t>С06</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="n"/>
-      <c r="Q7" s="7" t="n"/>
-      <c r="R7" s="7" t="n"/>
-      <c r="S7" s="7" t="n"/>
-      <c r="T7" s="7" t="n"/>
-      <c r="U7" s="7" t="n"/>
-      <c r="V7" s="7" t="n"/>
-      <c r="W7" s="7" t="n"/>
-      <c r="X7" s="7" t="n"/>
-      <c r="Y7" s="7" t="n"/>
-      <c r="Z7" s="7" t="n"/>
+      <c r="B7" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z7" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -4232,31 +4532,81 @@
           <t>С07</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
-      <c r="S8" s="7" t="n"/>
-      <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="n"/>
-      <c r="V8" s="7" t="n"/>
-      <c r="W8" s="7" t="n"/>
-      <c r="X8" s="7" t="n"/>
-      <c r="Y8" s="7" t="n"/>
-      <c r="Z8" s="7" t="n"/>
+      <c r="B8" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="P8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="T8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="X8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z8" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -4264,31 +4614,81 @@
           <t>С08</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="7" t="n"/>
-      <c r="Q9" s="7" t="n"/>
-      <c r="R9" s="7" t="n"/>
-      <c r="S9" s="7" t="n"/>
-      <c r="T9" s="7" t="n"/>
-      <c r="U9" s="7" t="n"/>
-      <c r="V9" s="7" t="n"/>
-      <c r="W9" s="7" t="n"/>
-      <c r="X9" s="7" t="n"/>
-      <c r="Y9" s="7" t="n"/>
-      <c r="Z9" s="7" t="n"/>
+      <c r="B9" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z9" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -4296,31 +4696,81 @@
           <t>С09</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
-      <c r="O10" s="7" t="n"/>
-      <c r="P10" s="7" t="n"/>
-      <c r="Q10" s="7" t="n"/>
-      <c r="R10" s="7" t="n"/>
-      <c r="S10" s="7" t="n"/>
-      <c r="T10" s="7" t="n"/>
-      <c r="U10" s="7" t="n"/>
-      <c r="V10" s="7" t="n"/>
-      <c r="W10" s="7" t="n"/>
-      <c r="X10" s="7" t="n"/>
-      <c r="Y10" s="7" t="n"/>
-      <c r="Z10" s="7" t="n"/>
+      <c r="B10" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="P10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z10" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -4328,31 +4778,81 @@
           <t>С10</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
-      <c r="O11" s="7" t="n"/>
-      <c r="P11" s="7" t="n"/>
-      <c r="Q11" s="7" t="n"/>
-      <c r="R11" s="7" t="n"/>
-      <c r="S11" s="7" t="n"/>
-      <c r="T11" s="7" t="n"/>
-      <c r="U11" s="7" t="n"/>
-      <c r="V11" s="7" t="n"/>
-      <c r="W11" s="7" t="n"/>
-      <c r="X11" s="7" t="n"/>
-      <c r="Y11" s="7" t="n"/>
-      <c r="Z11" s="7" t="n"/>
+      <c r="B11" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -4360,31 +4860,81 @@
           <t>С11</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="7" t="n"/>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
-      <c r="K12" s="7" t="n"/>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="n"/>
-      <c r="N12" s="7" t="n"/>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="7" t="n"/>
-      <c r="Q12" s="7" t="n"/>
-      <c r="R12" s="7" t="n"/>
-      <c r="S12" s="7" t="n"/>
-      <c r="T12" s="7" t="n"/>
-      <c r="U12" s="7" t="n"/>
-      <c r="V12" s="7" t="n"/>
-      <c r="W12" s="7" t="n"/>
-      <c r="X12" s="7" t="n"/>
-      <c r="Y12" s="7" t="n"/>
-      <c r="Z12" s="7" t="n"/>
+      <c r="B12" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z12" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -4392,31 +4942,81 @@
           <t>С12</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="7" t="n"/>
-      <c r="Q13" s="7" t="n"/>
-      <c r="R13" s="7" t="n"/>
-      <c r="S13" s="7" t="n"/>
-      <c r="T13" s="7" t="n"/>
-      <c r="U13" s="7" t="n"/>
-      <c r="V13" s="7" t="n"/>
-      <c r="W13" s="7" t="n"/>
-      <c r="X13" s="7" t="n"/>
-      <c r="Y13" s="7" t="n"/>
-      <c r="Z13" s="7" t="n"/>
+      <c r="B13" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="P13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="T13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="X13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z13" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -4424,31 +5024,81 @@
           <t>С13</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="7" t="n"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="n"/>
-      <c r="K14" s="7" t="n"/>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7" t="n"/>
-      <c r="N14" s="7" t="n"/>
-      <c r="O14" s="7" t="n"/>
-      <c r="P14" s="7" t="n"/>
-      <c r="Q14" s="7" t="n"/>
-      <c r="R14" s="7" t="n"/>
-      <c r="S14" s="7" t="n"/>
-      <c r="T14" s="7" t="n"/>
-      <c r="U14" s="7" t="n"/>
-      <c r="V14" s="7" t="n"/>
-      <c r="W14" s="7" t="n"/>
-      <c r="X14" s="7" t="n"/>
-      <c r="Y14" s="7" t="n"/>
-      <c r="Z14" s="7" t="n"/>
+      <c r="B14" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z14" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -4456,31 +5106,81 @@
           <t>С14</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="7" t="n"/>
-      <c r="I15" s="7" t="n"/>
-      <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
-      <c r="N15" s="7" t="n"/>
-      <c r="O15" s="7" t="n"/>
-      <c r="P15" s="7" t="n"/>
-      <c r="Q15" s="7" t="n"/>
-      <c r="R15" s="7" t="n"/>
-      <c r="S15" s="7" t="n"/>
-      <c r="T15" s="7" t="n"/>
-      <c r="U15" s="7" t="n"/>
-      <c r="V15" s="7" t="n"/>
-      <c r="W15" s="7" t="n"/>
-      <c r="X15" s="7" t="n"/>
-      <c r="Y15" s="7" t="n"/>
-      <c r="Z15" s="7" t="n"/>
+      <c r="B15" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="P15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="T15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="X15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z15" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -4488,31 +5188,81 @@
           <t>С15</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="7" t="n"/>
-      <c r="I16" s="7" t="n"/>
-      <c r="J16" s="7" t="n"/>
-      <c r="K16" s="7" t="n"/>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
-      <c r="N16" s="7" t="n"/>
-      <c r="O16" s="7" t="n"/>
-      <c r="P16" s="7" t="n"/>
-      <c r="Q16" s="7" t="n"/>
-      <c r="R16" s="7" t="n"/>
-      <c r="S16" s="7" t="n"/>
-      <c r="T16" s="7" t="n"/>
-      <c r="U16" s="7" t="n"/>
-      <c r="V16" s="7" t="n"/>
-      <c r="W16" s="7" t="n"/>
-      <c r="X16" s="7" t="n"/>
-      <c r="Y16" s="7" t="n"/>
-      <c r="Z16" s="7" t="n"/>
+      <c r="B16" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z16" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -4520,31 +5270,81 @@
           <t>С16</t>
         </is>
       </c>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
-      <c r="M17" s="7" t="n"/>
-      <c r="N17" s="7" t="n"/>
-      <c r="O17" s="7" t="n"/>
-      <c r="P17" s="7" t="n"/>
-      <c r="Q17" s="7" t="n"/>
-      <c r="R17" s="7" t="n"/>
-      <c r="S17" s="7" t="n"/>
-      <c r="T17" s="7" t="n"/>
-      <c r="U17" s="7" t="n"/>
-      <c r="V17" s="7" t="n"/>
-      <c r="W17" s="7" t="n"/>
-      <c r="X17" s="7" t="n"/>
-      <c r="Y17" s="7" t="n"/>
-      <c r="Z17" s="7" t="n"/>
+      <c r="B17" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="X17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z17" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -4552,31 +5352,81 @@
           <t>С17</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="n"/>
-      <c r="N18" s="7" t="n"/>
-      <c r="O18" s="7" t="n"/>
-      <c r="P18" s="7" t="n"/>
-      <c r="Q18" s="7" t="n"/>
-      <c r="R18" s="7" t="n"/>
-      <c r="S18" s="7" t="n"/>
-      <c r="T18" s="7" t="n"/>
-      <c r="U18" s="7" t="n"/>
-      <c r="V18" s="7" t="n"/>
-      <c r="W18" s="7" t="n"/>
-      <c r="X18" s="7" t="n"/>
-      <c r="Y18" s="7" t="n"/>
-      <c r="Z18" s="7" t="n"/>
+      <c r="B18" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U18" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z18" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -4584,31 +5434,81 @@
           <t>С18</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="7" t="n"/>
-      <c r="J19" s="7" t="n"/>
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
-      <c r="N19" s="7" t="n"/>
-      <c r="O19" s="7" t="n"/>
-      <c r="P19" s="7" t="n"/>
-      <c r="Q19" s="7" t="n"/>
-      <c r="R19" s="7" t="n"/>
-      <c r="S19" s="7" t="n"/>
-      <c r="T19" s="7" t="n"/>
-      <c r="U19" s="7" t="n"/>
-      <c r="V19" s="7" t="n"/>
-      <c r="W19" s="7" t="n"/>
-      <c r="X19" s="7" t="n"/>
-      <c r="Y19" s="7" t="n"/>
-      <c r="Z19" s="7" t="n"/>
+      <c r="B19" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -4616,31 +5516,81 @@
           <t>С19</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="n"/>
-      <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
-      <c r="O20" s="7" t="n"/>
-      <c r="P20" s="7" t="n"/>
-      <c r="Q20" s="7" t="n"/>
-      <c r="R20" s="7" t="n"/>
-      <c r="S20" s="7" t="n"/>
-      <c r="T20" s="7" t="n"/>
-      <c r="U20" s="7" t="n"/>
-      <c r="V20" s="7" t="n"/>
-      <c r="W20" s="7" t="n"/>
-      <c r="X20" s="7" t="n"/>
-      <c r="Y20" s="7" t="n"/>
-      <c r="Z20" s="7" t="n"/>
+      <c r="B20" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z20" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">

</xml_diff>